<commit_message>
sync 2026-03-18 01:35 | configs/config_importados.json,diagnosticos/config_importados_20260318_012457_fuzzy.csv,precios/lista_importados.xlsx,salidas/importados_precios.pdf
</commit_message>
<xml_diff>
--- a/precios/lista_importados.xlsx
+++ b/precios/lista_importados.xlsx
@@ -41,6 +41,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -62,11 +63,13 @@
       <color rgb="FFFFFFFF"/>
       <name val="Inter"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -122,19 +125,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -147,6 +150,29 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2A6099"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>

</xml_diff>